<commit_message>
Add function to compute dynamic keys Add actual files for Entony Soleil project
</commit_message>
<xml_diff>
--- a/DiagramUML.xlsx
+++ b/DiagramUML.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pro\Git\RepartKey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32A73BEB-E4F2-43C2-A792-4767099A2669}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2007E1C-879C-4C73-89DC-74D2B114DEFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9C2CFD62-ECDA-47A9-B5F1-6188C6239BA5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{9C2CFD62-ECDA-47A9-B5F1-6188C6239BA5}"/>
   </bookViews>
   <sheets>
-    <sheet name="Classes" sheetId="1" r:id="rId1"/>
+    <sheet name="UML Diagram" sheetId="1" r:id="rId1"/>
     <sheet name="StateMachine" sheetId="2" r:id="rId2"/>
+    <sheet name="Dynamic key" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="40">
   <si>
     <t>Consumer</t>
   </si>
@@ -110,12 +111,51 @@
   </si>
   <si>
     <t>state</t>
+  </si>
+  <si>
+    <t>Consommateur</t>
+  </si>
+  <si>
+    <t>Consommation</t>
+  </si>
+  <si>
+    <t>Ratio</t>
+  </si>
+  <si>
+    <t>P1</t>
+  </si>
+  <si>
+    <t>P2</t>
+  </si>
+  <si>
+    <t>C1</t>
+  </si>
+  <si>
+    <t>C2</t>
+  </si>
+  <si>
+    <t>C3</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
+  </si>
+  <si>
+    <t>Producteur</t>
+  </si>
+  <si>
+    <t>Production</t>
+  </si>
+  <si>
+    <t>Ratio conso/prod</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -205,12 +245,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1203,4 +1249,198 @@
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D160B451-286F-4F4E-B3AD-636D956B12B6}">
+  <dimension ref="B3:K14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" s="5">
+        <v>5</v>
+      </c>
+      <c r="D4" s="5">
+        <f>C4/C$7</f>
+        <v>0.5</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H4" s="6">
+        <f>$D4*$C$10*$C$14</f>
+        <v>3.333333333333333</v>
+      </c>
+      <c r="I4" s="6">
+        <f>$D4*$C$11*$C$14</f>
+        <v>1.6666666666666665</v>
+      </c>
+      <c r="J4" s="7">
+        <f>SUM(H4:I4)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B5" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5" s="5">
+        <v>3</v>
+      </c>
+      <c r="D5" s="5">
+        <f t="shared" ref="D5:D6" si="0">C5/C$7</f>
+        <v>0.3</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="H5" s="6">
+        <f t="shared" ref="H5:H6" si="1">$D5*$C$10*$C$14</f>
+        <v>2</v>
+      </c>
+      <c r="I5" s="6">
+        <f t="shared" ref="I5:I6" si="2">$D5*$C$11*$C$14</f>
+        <v>1</v>
+      </c>
+      <c r="J5" s="7">
+        <f t="shared" ref="J5:J6" si="3">SUM(H5:I5)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B6" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" s="5">
+        <v>2</v>
+      </c>
+      <c r="D6" s="5">
+        <f t="shared" si="0"/>
+        <v>0.2</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="H6" s="6">
+        <f t="shared" si="1"/>
+        <v>1.3333333333333333</v>
+      </c>
+      <c r="I6" s="6">
+        <f t="shared" si="2"/>
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="J6" s="7">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="K6" s="7">
+        <f>SUM(J4:J6)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B7" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" s="5">
+        <f>SUM(C4:C6)</f>
+        <v>10</v>
+      </c>
+      <c r="H7" s="7">
+        <f>SUM(H4:H6)</f>
+        <v>6.6666666666666661</v>
+      </c>
+      <c r="I7" s="7">
+        <f>SUM(I4:I6)</f>
+        <v>3.333333333333333</v>
+      </c>
+      <c r="J7" s="7"/>
+    </row>
+    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I8" s="7">
+        <f>SUM(H7:I7)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B9" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B10" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="5">
+        <v>10</v>
+      </c>
+      <c r="D10" s="8">
+        <f>C10/C$12</f>
+        <v>0.66666666666666663</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B11" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="5">
+        <v>5</v>
+      </c>
+      <c r="D11" s="8">
+        <f>C11/C$12</f>
+        <v>0.33333333333333331</v>
+      </c>
+    </row>
+    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B12" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" s="5">
+        <f>SUM(C10:C11)</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B14" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" s="10">
+        <f>IF(C7&gt;C12,1,C7/C12)</f>
+        <v>0.66666666666666663</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>